<commit_message>
update sub-dashboard to include knowledge graph schema and pipeline contract
</commit_message>
<xml_diff>
--- a/sub/TWRP C3B2 - Document Submittal Log.xlsx
+++ b/sub/TWRP C3B2 - Document Submittal Log.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uesholdings.sharepoint.com/sites/c3b2/Shared Documents/06-DC/01-MDL/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\frank\WorkBuddy\workbuddy\sub\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1670" documentId="13_ncr:1_{A01A6F68-F3B8-4F2B-A33E-2C4C83F82018}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8A32CE27-4813-4CCC-B6C6-169E58790799}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{748C7F3B-A160-4027-A088-06D2E5969FE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="602" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" tabRatio="602" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="4" r:id="rId1"/>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1218" uniqueCount="569">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1221" uniqueCount="571">
   <si>
     <t>Instructions to use MDL:</t>
   </si>
@@ -1773,6 +1773,12 @@
   </si>
   <si>
     <t>Approval Status present while Submission Status = NFS; or Resubmission Required = Yes while Submission Status ? {RTR,REJ}</t>
+  </si>
+  <si>
+    <t>Dashboard Title</t>
+  </si>
+  <si>
+    <t>Document Submittal Log</t>
   </si>
 </sst>
 </file>
@@ -1780,9 +1786,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="[$-14809]d\ mmm\ yyyy;@"/>
-    <numFmt numFmtId="165" formatCode="000000;"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="[$-14809]d\ mmm\ yyyy;@"/>
+    <numFmt numFmtId="166" formatCode="000000;"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -1928,7 +1934,7 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1972,19 +1978,19 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2033,16 +2039,16 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -2060,14 +2066,14 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -2088,7 +2094,7 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -42702,11 +42708,11 @@
       </c>
       <c r="L19" s="5">
         <f t="shared" ca="1" si="1"/>
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="M19" s="43">
         <f t="shared" ca="1" si="2"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N19" s="6" t="str" cm="1">
         <f t="array" ref="N19">_xlfn.IFS(
@@ -42750,11 +42756,11 @@
       </c>
       <c r="L20" s="5">
         <f t="shared" ca="1" si="1"/>
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="M20" s="43">
         <f t="shared" ca="1" si="2"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N20" s="6" t="str" cm="1">
         <f t="array" ref="N20">_xlfn.IFS(
@@ -42798,11 +42804,11 @@
       </c>
       <c r="L21" s="5">
         <f t="shared" ca="1" si="1"/>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="M21" s="43">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N21" s="6" t="str" cm="1">
         <f t="array" ref="N21">_xlfn.IFS(
@@ -42846,11 +42852,11 @@
       </c>
       <c r="L22" s="5">
         <f t="shared" ca="1" si="1"/>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M22" s="43">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N22" s="6" t="str" cm="1">
         <f t="array" ref="N22">_xlfn.IFS(
@@ -43924,11 +43930,11 @@
       </c>
       <c r="L41" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="M41" s="43">
         <f t="shared" ca="1" si="6"/>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="N41" s="6" t="str" cm="1">
         <f t="array" ref="N41">_xlfn.IFS(
@@ -43972,11 +43978,11 @@
       </c>
       <c r="L42" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="M42" s="43">
         <f t="shared" ca="1" si="6"/>
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="N42" s="6" t="str" cm="1">
         <f t="array" ref="N42">_xlfn.IFS(
@@ -44020,11 +44026,11 @@
       </c>
       <c r="L43" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="M43" s="43">
         <f t="shared" ca="1" si="6"/>
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="N43" s="6" t="str" cm="1">
         <f t="array" ref="N43">_xlfn.IFS(
@@ -44068,11 +44074,11 @@
       </c>
       <c r="L44" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M44" s="43">
         <f t="shared" ca="1" si="6"/>
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="N44" s="6" t="str" cm="1">
         <f t="array" ref="N44">_xlfn.IFS(
@@ -47813,11 +47819,11 @@
       </c>
       <c r="L112" s="5">
         <f t="shared" ca="1" si="15"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M112" s="43">
         <f t="shared" ref="M112" ca="1" si="17">L112-I112</f>
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="N112" s="6" t="str" cm="1">
         <f t="array" ref="N112">_xlfn.IFS(
@@ -48198,11 +48204,11 @@
       </c>
       <c r="L119" s="5">
         <f t="shared" ca="1" si="15"/>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="M119" s="43">
         <f t="shared" ca="1" si="16"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N119" s="6" t="str" cm="1">
         <f t="array" ref="N119">_xlfn.IFS(
@@ -48245,11 +48251,11 @@
       </c>
       <c r="L120" s="5">
         <f t="shared" ca="1" si="15"/>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="M120" s="43">
         <f t="shared" ca="1" si="16"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N120" s="6" t="str" cm="1">
         <f t="array" ref="N120">_xlfn.IFS(
@@ -48292,11 +48298,11 @@
       </c>
       <c r="L121" s="5">
         <f t="shared" ca="1" si="15"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="M121" s="43">
         <f t="shared" ca="1" si="16"/>
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="N121" s="6" t="str" cm="1">
         <f t="array" ref="N121">_xlfn.IFS(
@@ -48333,11 +48339,11 @@
       </c>
       <c r="L122" s="5">
         <f t="shared" ca="1" si="15"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M122" s="43">
         <f t="shared" ref="M122" ca="1" si="18">L122-I122</f>
-        <v>-13</v>
+        <v>-12</v>
       </c>
       <c r="N122" s="6" t="str" cm="1">
         <f t="array" ref="N122">_xlfn.IFS(
@@ -48380,11 +48386,11 @@
       </c>
       <c r="L123" s="5">
         <f t="shared" ca="1" si="15"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="M123" s="43">
         <f t="shared" ca="1" si="16"/>
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="N123" s="6" t="str" cm="1">
         <f t="array" ref="N123">_xlfn.IFS(
@@ -48421,11 +48427,11 @@
       </c>
       <c r="L124" s="5">
         <f t="shared" ca="1" si="15"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M124" s="43">
         <f t="shared" ref="M124" ca="1" si="19">L124-I124</f>
-        <v>-13</v>
+        <v>-12</v>
       </c>
       <c r="N124" s="6" t="str" cm="1">
         <f t="array" ref="N124">_xlfn.IFS(
@@ -48468,11 +48474,11 @@
       </c>
       <c r="L125" s="5">
         <f t="shared" ca="1" si="15"/>
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M125" s="43">
         <f t="shared" ca="1" si="16"/>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N125" s="6" t="str" cm="1">
         <f t="array" ref="N125">_xlfn.IFS(
@@ -48515,11 +48521,11 @@
       </c>
       <c r="L126" s="5">
         <f t="shared" ca="1" si="15"/>
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M126" s="43">
         <f t="shared" ca="1" si="16"/>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N126" s="6" t="str" cm="1">
         <f t="array" ref="N126">_xlfn.IFS(
@@ -48562,11 +48568,11 @@
       </c>
       <c r="L127" s="5">
         <f t="shared" ca="1" si="15"/>
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M127" s="43">
         <f t="shared" ca="1" si="16"/>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N127" s="6" t="str" cm="1">
         <f t="array" ref="N127">_xlfn.IFS(
@@ -48609,11 +48615,11 @@
       </c>
       <c r="L128" s="5">
         <f t="shared" ca="1" si="15"/>
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M128" s="43">
         <f t="shared" ca="1" si="16"/>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N128" s="6" t="str" cm="1">
         <f t="array" ref="N128">_xlfn.IFS(
@@ -48656,11 +48662,11 @@
       </c>
       <c r="L129" s="5">
         <f t="shared" ca="1" si="15"/>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M129" s="43">
         <f t="shared" ca="1" si="16"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N129" s="6" t="str" cm="1">
         <f t="array" ref="N129">_xlfn.IFS(
@@ -48703,11 +48709,11 @@
       </c>
       <c r="L130" s="5">
         <f t="shared" ca="1" si="15"/>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M130" s="43">
         <f t="shared" ca="1" si="16"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N130" s="6" t="str" cm="1">
         <f t="array" ref="N130">_xlfn.IFS(
@@ -48750,11 +48756,11 @@
       </c>
       <c r="L131" s="5">
         <f t="shared" ca="1" si="15"/>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M131" s="43">
         <f t="shared" ca="1" si="16"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N131" s="6" t="str" cm="1">
         <f t="array" ref="N131">_xlfn.IFS(
@@ -48797,11 +48803,11 @@
       </c>
       <c r="L132" s="5">
         <f t="shared" ref="L132:L200" ca="1" si="21">IF(NOT(ISBLANK($K132)),$K132-$H132,TODAY()-$H132)</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="M132" s="43">
         <f t="shared" ref="M132:M198" ca="1" si="22">L132-I132</f>
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="N132" s="6" t="str" cm="1">
         <f t="array" ref="N132">_xlfn.IFS(
@@ -48838,11 +48844,11 @@
       </c>
       <c r="L133" s="5">
         <f t="shared" ca="1" si="21"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M133" s="43">
         <f t="shared" ref="M133:M134" ca="1" si="23">L133-I133</f>
-        <v>-13</v>
+        <v>-12</v>
       </c>
       <c r="N133" s="6" t="str" cm="1">
         <f t="array" ref="N133">_xlfn.IFS(
@@ -48879,11 +48885,11 @@
       </c>
       <c r="L134" s="5">
         <f t="shared" ca="1" si="21"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M134" s="43">
         <f t="shared" ca="1" si="23"/>
-        <v>-20</v>
+        <v>-19</v>
       </c>
       <c r="N134" s="6" t="str" cm="1">
         <f t="array" ref="N134">_xlfn.IFS(
@@ -49150,11 +49156,11 @@
       </c>
       <c r="L139" s="5">
         <f t="shared" ca="1" si="21"/>
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="M139" s="43">
         <f t="shared" ca="1" si="22"/>
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N139" s="6" t="str" cm="1">
         <f t="array" ref="N139">_xlfn.IFS(
@@ -49197,11 +49203,11 @@
       </c>
       <c r="L140" s="5">
         <f t="shared" ca="1" si="21"/>
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="M140" s="43">
         <f t="shared" ca="1" si="22"/>
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N140" s="6" t="str" cm="1">
         <f t="array" ref="N140">_xlfn.IFS(
@@ -49244,11 +49250,11 @@
       </c>
       <c r="L141" s="5">
         <f t="shared" ca="1" si="21"/>
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="M141" s="43">
         <f t="shared" ca="1" si="22"/>
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N141" s="6" t="str" cm="1">
         <f t="array" ref="N141">_xlfn.IFS(
@@ -49291,11 +49297,11 @@
       </c>
       <c r="L142" s="5">
         <f t="shared" ca="1" si="21"/>
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="M142" s="43">
         <f t="shared" ca="1" si="22"/>
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N142" s="6" t="str" cm="1">
         <f t="array" ref="N142">_xlfn.IFS(
@@ -49338,11 +49344,11 @@
       </c>
       <c r="L143" s="5">
         <f t="shared" ca="1" si="21"/>
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="M143" s="43">
         <f t="shared" ca="1" si="22"/>
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N143" s="6" t="str" cm="1">
         <f t="array" ref="N143">_xlfn.IFS(
@@ -49385,11 +49391,11 @@
       </c>
       <c r="L144" s="5">
         <f t="shared" ca="1" si="21"/>
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="M144" s="43">
         <f t="shared" ca="1" si="22"/>
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N144" s="6" t="str" cm="1">
         <f t="array" ref="N144">_xlfn.IFS(
@@ -49432,11 +49438,11 @@
       </c>
       <c r="L145" s="5">
         <f t="shared" ca="1" si="21"/>
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="M145" s="43">
         <f t="shared" ca="1" si="22"/>
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N145" s="6" t="str" cm="1">
         <f t="array" ref="N145">_xlfn.IFS(
@@ -49479,11 +49485,11 @@
       </c>
       <c r="L146" s="5">
         <f t="shared" ca="1" si="21"/>
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="M146" s="43">
         <f t="shared" ca="1" si="22"/>
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N146" s="6" t="str" cm="1">
         <f t="array" ref="N146">_xlfn.IFS(
@@ -49526,11 +49532,11 @@
       </c>
       <c r="L147" s="5">
         <f t="shared" ca="1" si="21"/>
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="M147" s="43">
         <f t="shared" ca="1" si="22"/>
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N147" s="6" t="str" cm="1">
         <f t="array" ref="N147">_xlfn.IFS(
@@ -49573,11 +49579,11 @@
       </c>
       <c r="L148" s="5">
         <f t="shared" ca="1" si="21"/>
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="M148" s="43">
         <f t="shared" ca="1" si="22"/>
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N148" s="6" t="str" cm="1">
         <f t="array" ref="N148">_xlfn.IFS(
@@ -49620,11 +49626,11 @@
       </c>
       <c r="L149" s="5">
         <f t="shared" ca="1" si="21"/>
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="M149" s="43">
         <f t="shared" ca="1" si="22"/>
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N149" s="6" t="str" cm="1">
         <f t="array" ref="N149">_xlfn.IFS(
@@ -49667,11 +49673,11 @@
       </c>
       <c r="L150" s="5">
         <f t="shared" ca="1" si="21"/>
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="M150" s="43">
         <f t="shared" ca="1" si="22"/>
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N150" s="6" t="str" cm="1">
         <f t="array" ref="N150">_xlfn.IFS(
@@ -49714,11 +49720,11 @@
       </c>
       <c r="L151" s="5">
         <f t="shared" ca="1" si="21"/>
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="M151" s="43">
         <f t="shared" ca="1" si="22"/>
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N151" s="6" t="str" cm="1">
         <f t="array" ref="N151">_xlfn.IFS(
@@ -49761,11 +49767,11 @@
       </c>
       <c r="L152" s="5">
         <f t="shared" ca="1" si="21"/>
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="M152" s="43">
         <f t="shared" ca="1" si="22"/>
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N152" s="6" t="str" cm="1">
         <f t="array" ref="N152">_xlfn.IFS(
@@ -49808,11 +49814,11 @@
       </c>
       <c r="L153" s="5">
         <f t="shared" ca="1" si="21"/>
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="M153" s="43">
         <f t="shared" ca="1" si="22"/>
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N153" s="6" t="str" cm="1">
         <f t="array" ref="N153">_xlfn.IFS(
@@ -50070,11 +50076,11 @@
       </c>
       <c r="L187" s="5">
         <f t="shared" ca="1" si="21"/>
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="M187" s="43">
         <f t="shared" ca="1" si="22"/>
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="N187" s="6" t="str" cm="1">
         <f t="array" ref="N187">_xlfn.IFS(
@@ -50285,11 +50291,11 @@
       </c>
       <c r="L191" s="5">
         <f t="shared" ca="1" si="21"/>
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="M191" s="43">
         <f t="shared" ca="1" si="22"/>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="N191" s="6" t="str" cm="1">
         <f t="array" ref="N191">_xlfn.IFS(
@@ -50332,11 +50338,11 @@
       </c>
       <c r="L192" s="5">
         <f t="shared" ca="1" si="21"/>
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="M192" s="43">
         <f t="shared" ca="1" si="22"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="N192" s="6" t="str" cm="1">
         <f t="array" ref="N192">_xlfn.IFS(
@@ -50379,11 +50385,11 @@
       </c>
       <c r="L193" s="5">
         <f t="shared" ca="1" si="21"/>
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="M193" s="43">
         <f t="shared" ca="1" si="22"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="N193" s="6" t="str" cm="1">
         <f t="array" ref="N193">_xlfn.IFS(
@@ -50426,11 +50432,11 @@
       </c>
       <c r="L194" s="5">
         <f t="shared" ca="1" si="21"/>
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="M194" s="43">
         <f t="shared" ca="1" si="22"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="N194" s="6" t="str" cm="1">
         <f t="array" ref="N194">_xlfn.IFS(
@@ -50585,11 +50591,11 @@
       </c>
       <c r="L197" s="5">
         <f t="shared" ca="1" si="21"/>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="M197" s="43">
         <f t="shared" ca="1" si="22"/>
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="N197" s="6" t="str" cm="1">
         <f t="array" ref="N197">_xlfn.IFS(
@@ -50741,11 +50747,11 @@
       </c>
       <c r="L200" s="5">
         <f t="shared" ca="1" si="21"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="M200" s="43">
         <f t="shared" ca="1" si="24"/>
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="N200" s="6" t="str" cm="1">
         <f t="array" ref="N200">_xlfn.IFS(
@@ -51212,11 +51218,11 @@
       </c>
       <c r="L208" s="5">
         <f t="shared" ca="1" si="27"/>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="M208" s="43">
         <f t="shared" ref="M208" ca="1" si="29">L208-I208</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N208" s="6" t="str" cm="1">
         <f t="array" ref="N208">_xlfn.IFS(
@@ -51263,11 +51269,11 @@
       </c>
       <c r="L209" s="5">
         <f t="shared" ca="1" si="27"/>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="M209" s="43">
         <f t="shared" ca="1" si="28"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N209" s="6" t="str" cm="1">
         <f t="array" ref="N209">_xlfn.IFS(
@@ -51314,11 +51320,11 @@
       </c>
       <c r="L210" s="5">
         <f t="shared" ca="1" si="27"/>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="M210" s="43">
         <f t="shared" ca="1" si="28"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N210" s="6" t="str" cm="1">
         <f t="array" ref="N210">_xlfn.IFS(
@@ -51365,11 +51371,11 @@
       </c>
       <c r="L211" s="5">
         <f t="shared" ca="1" si="27"/>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="M211" s="43">
         <f t="shared" ref="M211:M212" ca="1" si="30">L211-I211</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N211" s="6" t="str" cm="1">
         <f t="array" ref="N211">_xlfn.IFS(
@@ -51416,11 +51422,11 @@
       </c>
       <c r="L212" s="5">
         <f t="shared" ca="1" si="27"/>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="M212" s="43">
         <f t="shared" ca="1" si="30"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N212" s="6" t="str" cm="1">
         <f t="array" ref="N212">_xlfn.IFS(
@@ -51587,11 +51593,11 @@
       </c>
       <c r="L215" s="5">
         <f t="shared" ca="1" si="27"/>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="M215" s="43">
         <f t="shared" ca="1" si="28"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N215" s="6" t="str" cm="1">
         <f t="array" ref="N215">_xlfn.IFS(
@@ -51989,11 +51995,11 @@
       </c>
       <c r="L224" s="5">
         <f t="shared" ca="1" si="32"/>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="M224" s="43">
         <f t="shared" ref="M224" ca="1" si="34">L224-I224</f>
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="N224" s="6" t="str" cm="1">
         <f t="array" ref="N224">_xlfn.IFS(
@@ -52328,7 +52334,7 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{817B8659-8FED-441E-8A24-629F29C2338D}">
           <x14:formula1>
-            <xm:f>Code!$B$9:$B$11</xm:f>
+            <xm:f>Code!$B$10:$B$12</xm:f>
           </x14:formula1>
           <xm:sqref>I92:I1048576 I2:I90</xm:sqref>
         </x14:dataValidation>
@@ -52350,7 +52356,7 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.1796875" customWidth="1"/>
     <col min="3" max="3" width="24.81640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21.26953125" bestFit="1" customWidth="1"/>
@@ -52538,13 +52544,13 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" s="7" t="s">
-        <v>477</v>
+        <v>569</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>478</v>
+        <v>570</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>479</v>
+        <v>449</v>
       </c>
       <c r="H6" s="37" t="s">
         <v>243</v>
@@ -52567,13 +52573,13 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" s="7" t="s">
-        <v>483</v>
-      </c>
-      <c r="B7" s="8">
-        <v>1</v>
+        <v>477</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>478</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>484</v>
+        <v>479</v>
       </c>
       <c r="H7" s="7"/>
       <c r="I7" s="7"/>
@@ -52592,10 +52598,10 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" s="7" t="s">
-        <v>487</v>
+        <v>483</v>
       </c>
       <c r="B8" s="8">
-        <v>20000</v>
+        <v>1</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>484</v>
@@ -52615,10 +52621,10 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" s="7" t="s">
-        <v>490</v>
-      </c>
-      <c r="B9" s="9">
-        <v>20</v>
+        <v>487</v>
+      </c>
+      <c r="B9" s="8">
+        <v>20000</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>484</v>
@@ -52638,10 +52644,10 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" s="7" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="B10" s="9">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>484</v>
@@ -52661,7 +52667,7 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" s="7" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="B11" s="9">
         <v>14</v>
@@ -52684,10 +52690,10 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>500</v>
+        <v>496</v>
+      </c>
+      <c r="B12" s="9">
+        <v>14</v>
       </c>
       <c r="C12" s="7" t="s">
         <v>484</v>
@@ -52707,13 +52713,13 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>449</v>
+        <v>484</v>
       </c>
       <c r="K13" s="7" t="s">
         <v>497</v>
@@ -52730,10 +52736,10 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="C14" s="7" t="s">
         <v>449</v>
@@ -52753,10 +52759,10 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>449</v>
@@ -52776,10 +52782,10 @@
     </row>
     <row r="16" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>513</v>
+        <v>509</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>449</v>
@@ -52799,10 +52805,10 @@
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A17" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>449</v>
@@ -52822,10 +52828,10 @@
     </row>
     <row r="18" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A18" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>520</v>
+        <v>516</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>449</v>
@@ -52845,13 +52851,13 @@
     </row>
     <row r="19" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>479</v>
+        <v>449</v>
       </c>
       <c r="K19" s="7" t="s">
         <v>517</v>
@@ -52868,13 +52874,13 @@
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A20" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>484</v>
+        <v>479</v>
       </c>
       <c r="K20" s="7" t="s">
         <v>514</v>
@@ -52891,13 +52897,13 @@
     </row>
     <row r="21" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>479</v>
+        <v>484</v>
       </c>
       <c r="K21" s="7" t="s">
         <v>527</v>
@@ -52914,10 +52920,10 @@
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A22" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="C22" s="7" t="s">
         <v>479</v>
@@ -52937,13 +52943,13 @@
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A23" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>536</v>
+        <v>532</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>484</v>
+        <v>479</v>
       </c>
       <c r="K23" s="7" t="s">
         <v>537</v>
@@ -52960,10 +52966,10 @@
     </row>
     <row r="24" spans="1:14" ht="58" x14ac:dyDescent="0.35">
       <c r="A24" s="7" t="s">
-        <v>539</v>
+        <v>28</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>540</v>
+        <v>536</v>
       </c>
       <c r="C24" s="7" t="s">
         <v>484</v>
@@ -52983,13 +52989,13 @@
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A25" s="7" t="s">
-        <v>31</v>
+        <v>539</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>449</v>
+        <v>484</v>
       </c>
       <c r="K25" s="7" t="s">
         <v>543</v>
@@ -53006,13 +53012,13 @@
     </row>
     <row r="26" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>546</v>
+        <v>542</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>547</v>
+        <v>449</v>
       </c>
       <c r="K26" s="7" t="s">
         <v>548</v>
@@ -53029,13 +53035,13 @@
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A27" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>551</v>
+        <v>546</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>449</v>
+        <v>547</v>
       </c>
       <c r="K27" s="7" t="s">
         <v>552</v>
@@ -53051,9 +53057,15 @@
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A28" s="7"/>
-      <c r="B28" s="7"/>
-      <c r="C28" s="7"/>
+      <c r="A28" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>551</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>449</v>
+      </c>
       <c r="K28" s="7" t="s">
         <v>555</v>
       </c>
@@ -53068,6 +53080,9 @@
       </c>
     </row>
     <row r="29" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+      <c r="A29" s="7"/>
+      <c r="B29" s="7"/>
+      <c r="C29" s="7"/>
       <c r="K29" s="7" t="s">
         <v>558</v>
       </c>
@@ -53135,6 +53150,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="dabe0c67-3730-4fa0-82e4-66182d905f97" xsi:nil="true"/>
@@ -53145,7 +53169,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010061E075E1F5F4354EAA6D40AAFDD7C5B7" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="413e7fbc6bfff51495b9935fab9c9eb7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d9e77098-5d25-4da0-8ec0-b428d9dfa13b" xmlns:ns3="dabe0c67-3730-4fa0-82e4-66182d905f97" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="72eddbe93d13f361e6527edddba36bff" ns2:_="" ns3:_="">
     <xsd:import namespace="d9e77098-5d25-4da0-8ec0-b428d9dfa13b"/>
@@ -53340,27 +53364,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{771E19F9-E9BE-4A38-A4E5-C2DC89D12BB3}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06A99400-7273-4660-B2DB-C8CE0A4C78EB}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="dabe0c67-3730-4fa0-82e4-66182d905f97"/>
-    <ds:schemaRef ds:uri="d9e77098-5d25-4da0-8ec0-b428d9dfa13b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{771E19F9-E9BE-4A38-A4E5-C2DC89D12BB3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="d9e77098-5d25-4da0-8ec0-b428d9dfa13b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="dabe0c67-3730-4fa0-82e4-66182d905f97"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0E007B31-40A9-49CA-A632-763EEED92CBC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -53377,12 +53406,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06A99400-7273-4660-B2DB-C8CE0A4C78EB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>